<commit_message>
Ajout de l'extension lieuDit (#165)
* replace precint

* update lieudit 3161f12ad8f3d935b0001d3c735a228231e9e1c9
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-as-address-extended.xlsx
+++ b/ig/main/StructureDefinition-as-address-extended.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-05T18:22:24+00:00</t>
+    <t>2024-02-05T18:22:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -600,20 +600,20 @@
     <t>The base name of a roadway or artery recognized by a municipality (excluding street type and direction).</t>
   </si>
   <si>
-    <t>Address.line.extension:precinct</t>
-  </si>
-  <si>
-    <t>precinct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {iso21090-ADXP-precinct}
+    <t>Address.line.extension:lieuDit</t>
+  </si>
+  <si>
+    <t>lieuDit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {https://interop.esante.gouv.fr/ig/fhir/annuaire/StructureDefinition/as-ext-lieu-dit}
 </t>
   </si>
   <si>
     <t>lieuDit (Adresse) : Lieu qui porte un nom rappelant une particularité topographique ou historique.</t>
   </si>
   <si>
-    <t>A subsection of a municipality.</t>
+    <t>Extension créée dans le cadre de l'Annuaire Santé pour indiquer le lieu dit</t>
   </si>
   <si>
     <t>Address.line.value</t>
@@ -1067,7 +1067,7 @@
     <col min="8" max="8" width="16.27734375" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="13.26171875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="75.0" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="86.08203125" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>